<commit_message>
Enhance BD project and follow-up models with new fields and update related logic
- Added `stage_changed_at` to `BDProject` to track stage changes.
- Introduced new fields in `BDFollowUp`: `outcome`, `outcome_code`, `completed_at`, `original_due_at`, and `snooze_count` for better follow-up management.
- Updated database migration logic to backfill new fields where necessary.
- Enhanced the `to_dict` method in `BDFollowUp` to include new fields in API responses.
- Improved follow-up handling in the admin routes, including reassignment and completion logic.
- Added new analytics constants for follow-up outcomes and statuses.

These changes aim to improve the tracking and management of projects and follow-ups within the BD module.
</commit_message>
<xml_diff>
--- a/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
+++ b/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
@@ -999,7 +999,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:47</t>
+          <t>Generated: 14 Sep 2026  17:23</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:47</t>
+          <t>Generated: 14 Sep 2026  17:23</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:47</t>
+          <t>Generated: 14 Sep 2026  17:23</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:47</t>
+          <t>Generated: 14 Sep 2026  17:23</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 05 Sep 2026  21:47</t>
+          <t>Generated: 14 Sep 2026  17:23</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Update application entry point from Injaaz.py to kynvera.py
- Renamed the main application file from Injaaz.py to kynvera.py to reflect the new structure.
- Updated all references throughout the codebase to ensure consistency with the new entry point.
- Enhanced documentation and scripts to reference kynvera.py for application startup and management.

These changes aim to streamline the application structure and improve clarity in the codebase.
</commit_message>
<xml_diff>
--- a/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
+++ b/\\172.25.70.143\Injaaz\General\CAFM/Daily Report on Resolved and Pending Complaints for 15th of July 2026 & 16th of July 2026.xlsx
@@ -999,7 +999,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 14 Sep 2026  17:23</t>
+          <t>Generated: 16 Sep 2026  13:14</t>
         </is>
       </c>
     </row>
@@ -1276,7 +1276,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 14 Sep 2026  17:23</t>
+          <t>Generated: 16 Sep 2026  13:14</t>
         </is>
       </c>
     </row>
@@ -1713,7 +1713,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 14 Sep 2026  17:23</t>
+          <t>Generated: 16 Sep 2026  13:14</t>
         </is>
       </c>
     </row>
@@ -1974,7 +1974,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 14 Sep 2026  17:23</t>
+          <t>Generated: 16 Sep 2026  13:14</t>
         </is>
       </c>
     </row>
@@ -2104,7 +2104,7 @@
     <row r="3" ht="18" customHeight="1">
       <c r="B3" s="3" t="inlineStr">
         <is>
-          <t>Generated: 14 Sep 2026  17:23</t>
+          <t>Generated: 16 Sep 2026  13:14</t>
         </is>
       </c>
     </row>

</xml_diff>